<commit_message>
Tavolo base: traversa bassa anteriore cassetti (ACi) e viste ortogonali quotate
- Aggiunta traversa ACi tra G1A e G2A: 5 barre KVH, fori derivati dal modello
- Tavole e manuale: pianta telaio, prospetti, fianchi, pianta piano, schede
  quotate delle traverse
- Quantità ferramenta e costi aggiornati

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014ifKLy6ksUu35M7vyqXshy
</commit_message>
<xml_diff>
--- a/moduli/1-tavolo-base/tavolo_base_costi.xlsx
+++ b/moduli/1-tavolo-base/tavolo_base_costi.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="135">
   <si>
     <t xml:space="preserve">Modulo 1 – Tavolo base: distinta e costi</t>
   </si>
@@ -61,7 +61,7 @@
     <t xml:space="preserve">Trave KVH giuntato 80×120, barra 4 m</t>
   </si>
   <si>
-    <t xml:space="preserve">gambe, traverse e i 4 montanti dell'alzatina (schema senza scorta)</t>
+    <t xml:space="preserve">gambe, traverse e i 4 montanti dell'alzatina (~2,6 m di scorta)</t>
   </si>
   <si>
     <t xml:space="preserve">pz</t>
@@ -106,13 +106,13 @@
     <t xml:space="preserve">Bullone TCEI M10×140 + rondella Ø20 (B2)</t>
   </si>
   <si>
-    <t xml:space="preserve">traverse longitudinali, gambe d'estremità</t>
+    <t xml:space="preserve">traverse longitudinali, gambe con una sola traversa</t>
   </si>
   <si>
     <t xml:space="preserve">Dado a tamburo M10 (D)</t>
   </si>
   <si>
-    <t xml:space="preserve">32 nodi + 4 predisposizione alzatina</t>
+    <t xml:space="preserve">34 nodi + 4 predisposizione alzatina</t>
   </si>
   <si>
     <t xml:space="preserve">Barra filettata M10 da 1 m (R)</t>
@@ -400,19 +400,31 @@
     <t xml:space="preserve">Barra 1</t>
   </si>
   <si>
-    <t xml:space="preserve">700 + 700 + 700 + 700 + 560 + 500</t>
+    <t xml:space="preserve">700 + 700 + 700 + 560 + 500 + 500</t>
   </si>
   <si>
     <t xml:space="preserve">Barra 2</t>
   </si>
   <si>
+    <t xml:space="preserve">700 + 700 + 560 + 560 + 560 + 500</t>
+  </si>
+  <si>
     <t xml:space="preserve">Barra 3</t>
   </si>
   <si>
-    <t xml:space="preserve">700 + 560 + 560 + 560 + 480 + 480 + 250 + 250</t>
+    <t xml:space="preserve">700 + 700 + 700 + 560 + 480 + 480</t>
   </si>
   <si>
     <t xml:space="preserve">Barra 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">700 + 700</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barra 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">560 + 560 + 560 + 480 + 480 + 250 + 250 + 250 + 250</t>
   </si>
   <si>
     <t xml:space="preserve">I 4 pezzi da 250 sono i montanti dell'alzatina: tagliali e conservali anche se l'alzatina la farai dopo.</t>
@@ -1005,7 +1017,7 @@
       </c>
       <c r="D5" s="6" t="n">
         <f aca="false">'Confronto travi'!I8</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>13</v>
@@ -1016,7 +1028,7 @@
       </c>
       <c r="G5" s="8" t="n">
         <f aca="false">D5*F5</f>
-        <v>119.6</v>
+        <v>149.5</v>
       </c>
       <c r="H5" s="5" t="s">
         <v>14</v>
@@ -1141,7 +1153,7 @@
         <v>27</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>13</v>
@@ -1151,7 +1163,7 @@
       </c>
       <c r="G10" s="8" t="n">
         <f aca="false">D10*F10</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H10" s="5" t="s">
         <v>22</v>
@@ -1168,7 +1180,7 @@
         <v>29</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>13</v>
@@ -1178,7 +1190,7 @@
       </c>
       <c r="G11" s="8" t="n">
         <f aca="false">D11*F11</f>
-        <v>28.8</v>
+        <v>30.4</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>22</v>
@@ -1595,7 +1607,7 @@
       </c>
       <c r="G28" s="8" t="n">
         <f aca="false">SUMIFS(G5:G26,H5:H26,"fornito da te")+SUMIFS(G5:G26,H5:H26,"OBI, verificato 18/10/2026")</f>
-        <v>230.09</v>
+        <v>259.99</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1604,7 +1616,7 @@
       </c>
       <c r="G29" s="8" t="n">
         <f aca="false">SUMIFS(G5:G26,H5:H26,"stima – da verificare")</f>
-        <v>359.1</v>
+        <v>362.7</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1613,7 +1625,7 @@
       </c>
       <c r="G30" s="14" t="n">
         <f aca="false">SUM(G5:G26)</f>
-        <v>589.19</v>
+        <v>622.69</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1622,7 +1634,7 @@
       </c>
       <c r="G32" s="8" t="n">
         <f aca="false">SUMIFS(G5:G26,A5:A26,"Legno")</f>
-        <v>240.09</v>
+        <v>269.99</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1631,7 +1643,7 @@
       </c>
       <c r="G33" s="8" t="n">
         <f aca="false">SUMIFS(G5:G26,A5:A26,"Ferramenta telaio")</f>
-        <v>139.1</v>
+        <v>142.7</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1754,7 +1766,7 @@
         <v>13.9166666666667</v>
       </c>
       <c r="F5" s="17" t="n">
-        <v>14.76</v>
+        <v>15.26</v>
       </c>
       <c r="G5" s="15" t="n">
         <v>5.1</v>
@@ -1785,7 +1797,7 @@
         <v>13.975</v>
       </c>
       <c r="F6" s="17" t="n">
-        <v>14.76</v>
+        <v>15.26</v>
       </c>
       <c r="G6" s="15" t="n">
         <v>5.1</v>
@@ -1816,17 +1828,17 @@
         <v>7.975</v>
       </c>
       <c r="F7" s="17" t="n">
-        <v>15.72</v>
+        <v>16.22</v>
       </c>
       <c r="G7" s="15" t="n">
         <v>1.6</v>
       </c>
       <c r="I7" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J7" s="8" t="n">
         <f aca="false">I7*D7</f>
-        <v>127.6</v>
+        <v>159.5</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1847,18 +1859,18 @@
         <v>7.475</v>
       </c>
       <c r="F8" s="23" t="n">
-        <v>15.4</v>
+        <v>15.9</v>
       </c>
       <c r="G8" s="20" t="n">
         <v>3.4</v>
       </c>
       <c r="H8" s="24"/>
       <c r="I8" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J8" s="26" t="n">
         <f aca="false">I8*D8</f>
-        <v>119.6</v>
+        <v>149.5</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1879,7 +1891,7 @@
         <v>9.975</v>
       </c>
       <c r="F9" s="17" t="n">
-        <v>15.08</v>
+        <v>15.58</v>
       </c>
       <c r="G9" s="15" t="n">
         <v>4.2</v>
@@ -2098,11 +2110,11 @@
         <v>125</v>
       </c>
       <c r="C4" s="28" t="n">
-        <v>3894</v>
+        <v>3694</v>
       </c>
       <c r="D4" s="29" t="n">
         <f aca="false">4000-C4</f>
-        <v>106</v>
+        <v>306</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2110,49 +2122,64 @@
         <v>126</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C5" s="28" t="n">
-        <v>3894</v>
+        <v>3614</v>
       </c>
       <c r="D5" s="29" t="n">
         <f aca="false">4000-C5</f>
-        <v>106</v>
+        <v>386</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C6" s="28" t="n">
-        <v>3882</v>
+        <v>3654</v>
       </c>
       <c r="D6" s="29" t="n">
         <f aca="false">4000-C6</f>
-        <v>118</v>
+        <v>346</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C7" s="28" t="n">
-        <v>3882</v>
+        <v>1418</v>
       </c>
       <c r="D7" s="29" t="n">
         <f aca="false">4000-C7</f>
-        <v>118</v>
+        <v>2582</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="C8" s="28" t="n">
+        <v>3686</v>
+      </c>
+      <c r="D8" s="29" t="n">
+        <f aca="false">4000-C8</f>
+        <v>314</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Prezzi verificati su Tecnomat, OBI e Leroy Merlin; mensola in tavole 1000x200x18
- Fogli costi con negozio, prezzo verificato e link per ogni voce
- Nuovo confronto_prezzi_negozi.xlsx con giunzioni alternative
- Alzatina: tavole lamellari 1000x200x18 Tecnomat al posto delle OBI 800x200x14
- Cassettiera: pannelli pretagliati 1200x600 e fibra 3 mm, schema di taglio aggiornato
- Manuali: nomi della ferramenta disponibile in negozio

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014ifKLy6ksUu35M7vyqXshy
</commit_message>
<xml_diff>
--- a/moduli/1-tavolo-base/tavolo_base_costi.xlsx
+++ b/moduli/1-tavolo-base/tavolo_base_costi.xlsx
@@ -23,18 +23,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="169">
   <si>
     <t xml:space="preserve">Modulo 1 – Tavolo base: distinta e costi</t>
   </si>
   <si>
-    <t xml:space="preserve">Celle gialle = stime da sostituire con i prezzi reali. Testo blu = dato modificabile, verde = collegato a un altro foglio.</t>
+    <t xml:space="preserve">Prezzi verificati sui siti di Tecnomat, OBI e Leroy Merlin il 18/10/2026 (possono variare per negozio). Celle gialle = stime.</t>
   </si>
   <si>
     <t xml:space="preserve">Categoria</t>
   </si>
   <si>
-    <t xml:space="preserve">Articolo</t>
+    <t xml:space="preserve">Articolo (prodotto trovato)</t>
   </si>
   <si>
     <t xml:space="preserve">Uso</t>
@@ -55,10 +55,19 @@
     <t xml:space="preserve">Fonte prezzo</t>
   </si>
   <si>
+    <t xml:space="preserve">Negozio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Link</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note</t>
+  </si>
+  <si>
     <t xml:space="preserve">Legno</t>
   </si>
   <si>
-    <t xml:space="preserve">Trave KVH giuntato 80×120, barra 4 m</t>
+    <t xml:space="preserve">Trave legno massiccio strutturale KVH giuntato 80×120×4000</t>
   </si>
   <si>
     <t xml:space="preserve">gambe, traverse e i 4 montanti dell'alzatina (~2,6 m di scorta)</t>
@@ -67,7 +76,16 @@
     <t xml:space="preserve">pz</t>
   </si>
   <si>
-    <t xml:space="preserve">fornito da te</t>
+    <t xml:space="preserve">verificato 18/10/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tecnomat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">apri</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solo Tecnomat; OBI e Leroy Merlin non hanno KVH</t>
   </si>
   <si>
     <t xml:space="preserve">Tavola abete lamellare 2000×800×40</t>
@@ -76,79 +94,118 @@
     <t xml:space="preserve">piano di lavoro (intero)</t>
   </si>
   <si>
-    <t xml:space="preserve">Pannello OSB/3 2500×1250×18</t>
+    <t xml:space="preserve">Leroy Merlin: 147,45 € (marketplace); OBI: non c'è lo spessore 40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OSB 3 pioppo 18 mm 2500×1250</t>
   </si>
   <si>
     <t xml:space="preserve">3 ripiani bassi + rinforzo ricarica (2 strati)</t>
   </si>
   <si>
-    <t xml:space="preserve">OBI, verificato 18/10/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Listello abete 30×40, barra 2,4 m</t>
+    <t xml:space="preserve">OBI 31,49 €, Leroy Merlin 30,50 €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Listello abete grezzo 30×40×2000</t>
   </si>
   <si>
     <t xml:space="preserve">reggiripiano: 4 × 560 + 2 × 260</t>
   </si>
   <si>
+    <t xml:space="preserve">Grezzo va bene: resta nascosto sotto i ripiani</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ferramenta telaio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vite a testa cilindrica zincata M10×180 (B1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">traverse laterali</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OBI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In negozio verifica che sia a esagono incassato (TCEI); TCEI M10×180 non trovate a scaffale altrove</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viti a testa cilindrica M10×160, conf. 10 pz (B2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">traverse longitudinali</t>
+  </si>
+  <si>
+    <t xml:space="preserve">conf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accorciale a 140 mm con il seghetto (avvita prima un dado per ripulire il filetto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dado a tamburo M10 (D)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">34 nodi + 4 predisposizione alzatina</t>
+  </si>
+  <si>
     <t xml:space="preserve">stima – da verificare</t>
   </si>
   <si>
-    <t xml:space="preserve">Ferramenta telaio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bullone TCEI M10×180 + rondella Ø20 (B1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">traverse laterali</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bullone TCEI M10×140 + rondella Ø20 (B2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">traverse longitudinali, gambe con una sola traversa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dado a tamburo M10 (D)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">34 nodi + 4 predisposizione alzatina</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Barra filettata M10 da 1 m (R)</t>
+    <t xml:space="preserve">ferramenta/online</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non venduto dai tre negozi: ferramenta, Würth o online. Misura il diametro prima di forare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barra filettata M10×1000 zincata (R)</t>
   </si>
   <si>
     <t xml:space="preserve">4 spezzoni da 220 per le gambe centrali</t>
   </si>
   <si>
-    <t xml:space="preserve">Spine in faggio Ø12×50 (conf. 100)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 per nodo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">conf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Colla vinilica D3 750 g</t>
+    <t xml:space="preserve">OBI 3,19 €, LM 1,75 €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spine in faggio zigrinato Ø12, conf. 25 pz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 per testata (68)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lunghezza non indicata: servono ~50 mm. In alternativa tondo faggio Ø12×1000 Tecnomat 0,80 € da tagliare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collante vinilico D3 Tover 500 ml</t>
   </si>
   <si>
     <t xml:space="preserve">spine, rinforzo, listelli</t>
   </si>
   <si>
-    <t xml:space="preserve">Inserto filettato M10 + piedino livellatore</t>
+    <t xml:space="preserve">Piede regolabile Ø40 vite M10, conf. 2 pz</t>
   </si>
   <si>
     <t xml:space="preserve">sotto le gambe</t>
   </si>
   <si>
-    <t xml:space="preserve">Squadrette con asola + viti</t>
+    <t xml:space="preserve">Dado ragno M10 zincato (al posto dell'inserto a vite)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sede filettata sotto ogni gamba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Foro Ø12 invece di Ø14; pezzi per confezione non indicati. Inserti M10 a vite: solo marketplace LM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Squadretta a L 30×38×30 zincata</t>
   </si>
   <si>
     <t xml:space="preserve">fissaggio del piano</t>
   </si>
   <si>
-    <t xml:space="preserve">Viti assortite (5×60, 5×70, 4×50, 4,5×25)</t>
+    <t xml:space="preserve">Senza asola: allunga a mano il foro verso il piano con una punta Ø6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viti legno assortite (5×60, 5×70, 4×35, 4×50, 4,5×25)</t>
   </si>
   <si>
     <t xml:space="preserve">rinforzo, listelli, ripiani, squadrette</t>
@@ -157,12 +214,18 @@
     <t xml:space="preserve">set</t>
   </si>
   <si>
-    <t xml:space="preserve">Angolare a L 100×100 + tassello Ø8</t>
+    <t xml:space="preserve">Staffa angolare con nervatura 90×90×65 zincata</t>
   </si>
   <si>
     <t xml:space="preserve">fissaggio a muro (G1P e G4P)</t>
   </si>
   <si>
+    <t xml:space="preserve">Tasselli Ø8 per il tipo di muro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fissaggio a muro</t>
+  </si>
+  <si>
     <t xml:space="preserve">Zona ricarica</t>
   </si>
   <si>
@@ -175,18 +238,42 @@
     <t xml:space="preserve">lotto</t>
   </si>
   <si>
-    <t xml:space="preserve">Viti TSPEI M10×110 + rondella larga + dado autobloccante</t>
+    <t xml:space="preserve">officina/carpenteria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chiedi un preventivo a un'officina o a un servizio di taglio laser</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vite TSPEI M10×110 + dado autobloccante</t>
   </si>
   <si>
     <t xml:space="preserve">base, 2 posteriori</t>
   </si>
   <si>
-    <t xml:space="preserve">Viti TSPEI M10×200 + rondella larga + dado autobloccante</t>
+    <t xml:space="preserve">Non trovate a scaffale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vite TSPEI M10×200 + dado autobloccante</t>
   </si>
   <si>
     <t xml:space="preserve">base, 2 anteriori</t>
   </si>
   <si>
+    <t xml:space="preserve">Dadi autobloccanti M10 inox, conf. 10 pz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sotto la base</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rondelle piane larghe M10 (Ø29,5), conf. 8 pz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sotto la traversa e la contropiastra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leroy Merlin</t>
+  </si>
+  <si>
     <t xml:space="preserve">Manopole a stella M12 + 2 spine Ø10 h8</t>
   </si>
   <si>
@@ -199,13 +286,16 @@
     <t xml:space="preserve">Elettrico</t>
   </si>
   <si>
-    <t xml:space="preserve">Canalina passacavi sottoscrivania</t>
-  </si>
-  <si>
-    <t xml:space="preserve">una per campata</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Passacavi Ø60 da incasso</t>
+    <t xml:space="preserve">Canalina di distribuzione Arnocanali 60×40, 2 scomparti</t>
+  </si>
+  <si>
+    <t xml:space="preserve">una per campata (da tagliare)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lunghezza non indicata: verifica. Alternativa specifica sottoscrivania: LM 76 cm 36,95 € (online)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bocchette passacavi Ø60 PVC nero, conf. 2 pz</t>
   </si>
   <si>
     <t xml:space="preserve">piano</t>
@@ -220,10 +310,22 @@
     <t xml:space="preserve">Finitura</t>
   </si>
   <si>
-    <t xml:space="preserve">Olio/impregnante 750 ml + abrasivi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">telaio e piano; vernice trasparente per l'OSB</t>
+    <t xml:space="preserve">Olio Adler facile applicazione interno 750 ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">piano di lavoro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Impregnante legno all'acqua Cipir 0,75 l incolore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">telaio e ripiani OSB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abrasivi 80–120–180</t>
+  </si>
+  <si>
+    <t xml:space="preserve">levigatura</t>
   </si>
   <si>
     <t xml:space="preserve">Prezzi verificati</t>
@@ -250,10 +352,28 @@
     <t xml:space="preserve">di cui finitura</t>
   </si>
   <si>
-    <t xml:space="preserve">Travi e lamellare: prezzi forniti da te. OSB/3 18: prezzo OBI verificato il 18/10/2026. Il resto sono stime.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">I 4 dadi a tamburo della predisposizione vanno inseriti durante il montaggio: con il tavolo a muro non si raggiungono.</t>
+    <t xml:space="preserve">da Leroy Merlin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">da OBI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">da Tecnomat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">da ferramenta/online</t>
+  </si>
+  <si>
+    <t xml:space="preserve">da officina/carpenteria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tecnomat: taglio legno in negozio, 1° taglio gratis poi 1 € a taglio (solo per pannelli e listelli comprati lì).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I prezzi Tecnomat sono del negozio predefinito del sito (Roma Prenestina): controlla quello dove andrai.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I 4 dadi a tamburo della predisposizione alzatina vanno inseriti durante il montaggio del tavolo.</t>
   </si>
   <si>
     <t xml:space="preserve">Confronto travi per il telaio</t>
@@ -313,13 +433,10 @@
     <t xml:space="preserve">100×120</t>
   </si>
   <si>
-    <t xml:space="preserve">Riga verde = trave scelta. Barre calcolate con ottimizzazione del taglio (foglio 'Taglio travi').</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ripiani bassi e rinforzo ricarica: tre materiali a confronto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Servono: ripiano cassetti 500×560, ripiano ricarica 480×560, ripiano seduta 700×260, rinforzo 480×520 (spessore ≥ 36).</t>
+    <t xml:space="preserve">Riga verde = trave scelta (Tecnomat). Lamellare GL24h 80×120×4000 Tecnomat 39,90 €; Leroy Merlin 74,90–79,90 €; OBI non ha travi 80×120.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ripiani bassi e rinforzo ricarica: materiali a confronto</t>
   </si>
   <si>
     <t xml:space="preserve">Materiale</t>
@@ -328,31 +445,25 @@
     <t xml:space="preserve">Formato</t>
   </si>
   <si>
-    <t xml:space="preserve">Spessore ripiani</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pezzi necessari</t>
+    <t xml:space="preserve">Pezzi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prezzo</t>
   </si>
   <si>
     <t xml:space="preserve">Costo</t>
   </si>
   <si>
-    <t xml:space="preserve">Fonte</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Note</t>
-  </si>
-  <si>
     <t xml:space="preserve">OSB/3 18 (SCELTO)</t>
   </si>
   <si>
     <t xml:space="preserve">2500×1250</t>
   </si>
   <si>
-    <t xml:space="preserve">18 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Un pannello per tutto: 3 ripiani + rinforzo in 2 strati (36 mm). Avanzano ~1,8 m² (utili anche per la cassettiera).</t>
+    <t xml:space="preserve">Un pannello per 3 ripiani + rinforzo in 2 strati; avanzano ~1,8 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OSB/3 18</t>
   </si>
   <si>
     <t xml:space="preserve">Lamellare abete 40</t>
@@ -361,25 +472,16 @@
     <t xml:space="preserve">2000×800</t>
   </si>
   <si>
-    <t xml:space="preserve">40 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Un pannello per tutto, ripiani più spessi e belli; costa 2,5 volte l'OSB.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tavola OBI lamellare 14</t>
+    <t xml:space="preserve">Ripiani più spessi e belli, 2,9 volte l'OSB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tavola lamellare 14</t>
   </si>
   <si>
     <t xml:space="preserve">800×200</t>
   </si>
   <si>
-    <t xml:space="preserve">14 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8 tavole per i ripiani (3 + 3 + 2, una tagliata in larghezza) + 6 per il rinforzo in 2 strati da 28 mm. La più cara e la più sottile.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Costo al m²: OSB 18 ≈ 10 €/m² · lamellare 40 ≈ 49 €/m² · tavola OBI 14 ≈ 51 €/m².</t>
+    <t xml:space="preserve">8 per i ripiani + 6 per il rinforzo: la più cara</t>
   </si>
   <si>
     <t xml:space="preserve">Taglio travi KVH 80×120 (barre da 4 m)</t>
@@ -427,7 +529,7 @@
     <t xml:space="preserve">560 + 560 + 560 + 480 + 480 + 250 + 250 + 250 + 250</t>
   </si>
   <si>
-    <t xml:space="preserve">I 4 pezzi da 250 sono i montanti dell'alzatina: tagliali e conservali anche se l'alzatina la farai dopo.</t>
+    <t xml:space="preserve">I 4 pezzi da 250 sono i montanti dell'alzatina: tagliali e conservali. Tecnomat taglia in negozio (1 € a taglio dopo il primo).</t>
   </si>
 </sst>
 </file>
@@ -443,7 +545,7 @@
     <numFmt numFmtId="169" formatCode="0.00"/>
     <numFmt numFmtId="170" formatCode="#,##0"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -497,6 +599,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FF008000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <u val="single"/>
+      <sz val="11"/>
+      <color rgb="FF1F5FA8"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -584,7 +694,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -621,15 +731,19 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -645,7 +759,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -653,7 +767,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -665,11 +779,11 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -677,7 +791,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -685,7 +799,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -697,7 +811,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -738,7 +852,7 @@
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FF1F5FA8"/>
       <rgbColor rgb="FFCCCCFF"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
@@ -957,16 +1071,19 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:K52"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="46"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1004,23 +1121,32 @@
       <c r="H4" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="I4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D5" s="6" t="n">
         <f aca="false">'Confronto travi'!I8</f>
         <v>5</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F5" s="7" t="n">
         <f aca="false">'Confronto travi'!D8</f>
@@ -1031,26 +1157,35 @@
         <v>149.5</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>17</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J5" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C6" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" s="10" t="n">
+      <c r="F6" s="11" t="n">
         <v>79</v>
       </c>
       <c r="G6" s="8" t="n">
@@ -1058,134 +1193,179 @@
         <v>79</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>17</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J6" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="D7" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" s="10" t="n">
-        <v>31.49</v>
+        <v>16</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>27.5</v>
       </c>
       <c r="G7" s="8" t="n">
         <f aca="false">D7*F7</f>
-        <v>31.49</v>
+        <v>27.5</v>
       </c>
       <c r="H7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J7" s="9" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="K7" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="9" t="n">
+        <v>28</v>
+      </c>
+      <c r="D8" s="10" t="n">
         <v>2</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F8" s="11" t="n">
-        <v>5</v>
+        <v>3.1</v>
       </c>
       <c r="G8" s="8" t="n">
         <f aca="false">D8*F8</f>
-        <v>10</v>
+        <v>6.2</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>17</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J8" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="D9" s="9" t="n">
+        <v>32</v>
+      </c>
+      <c r="D9" s="10" t="n">
         <v>16</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>1.2</v>
+        <v>1.39</v>
       </c>
       <c r="G9" s="8" t="n">
         <f aca="false">D9*F9</f>
-        <v>19.2</v>
+        <v>22.24</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>17</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J9" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" s="9" t="n">
-        <v>10</v>
+        <v>36</v>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="F10" s="11" t="n">
-        <v>1</v>
+        <v>13.09</v>
       </c>
       <c r="G10" s="8" t="n">
         <f aca="false">D10*F10</f>
-        <v>10</v>
+        <v>13.09</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>17</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J10" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="D11" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="D11" s="10" t="n">
         <v>38</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F11" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="F11" s="12" t="n">
         <v>0.8</v>
       </c>
       <c r="G11" s="8" t="n">
@@ -1193,497 +1373,884 @@
         <v>30.4</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>41</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="J11" s="4"/>
+      <c r="K11" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="D12" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="D12" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F12" s="11" t="n">
-        <v>3.5</v>
+        <v>1.65</v>
       </c>
       <c r="G12" s="8" t="n">
         <f aca="false">D12*F12</f>
-        <v>3.5</v>
+        <v>1.65</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>17</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J12" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D13" s="9" t="n">
-        <v>1</v>
+        <v>48</v>
+      </c>
+      <c r="D13" s="10" t="n">
+        <v>3</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="F13" s="11" t="n">
-        <v>6</v>
+        <v>3.69</v>
       </c>
       <c r="G13" s="8" t="n">
         <f aca="false">D13*F13</f>
-        <v>6</v>
+        <v>11.07</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>17</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J13" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D14" s="9" t="n">
+        <v>51</v>
+      </c>
+      <c r="D14" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F14" s="11" t="n">
-        <v>9</v>
+        <v>4.95</v>
       </c>
       <c r="G14" s="8" t="n">
         <f aca="false">D14*F14</f>
-        <v>9</v>
+        <v>4.95</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>17</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J14" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K14" s="5"/>
+    </row>
+    <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="B15" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E15" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C15" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="D15" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>13</v>
-      </c>
       <c r="F15" s="11" t="n">
-        <v>3</v>
+        <v>1.65</v>
       </c>
       <c r="G15" s="8" t="n">
         <f aca="false">D15*F15</f>
-        <v>24</v>
+        <v>6.6</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>17</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J15" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K15" s="5"/>
+    </row>
+    <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="D16" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="E16" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E16" s="4" t="s">
-        <v>13</v>
-      </c>
       <c r="F16" s="11" t="n">
-        <v>0.6</v>
+        <v>2.79</v>
       </c>
       <c r="G16" s="8" t="n">
         <f aca="false">D16*F16</f>
-        <v>9.6</v>
+        <v>22.32</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>17</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J16" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K16" s="5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="D17" s="9" t="n">
-        <v>1</v>
+        <v>58</v>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>16</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>43</v>
+        <v>16</v>
       </c>
       <c r="F17" s="11" t="n">
-        <v>15</v>
+        <v>0.5</v>
       </c>
       <c r="G17" s="8" t="n">
         <f aca="false">D17*F17</f>
+        <v>8</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J17" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K17" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="F18" s="12" t="n">
         <v>15</v>
-      </c>
-      <c r="H17" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="D18" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F18" s="11" t="n">
-        <v>4</v>
       </c>
       <c r="G18" s="8" t="n">
         <f aca="false">D18*F18</f>
+        <v>15</v>
+      </c>
+      <c r="H18" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="I18" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J18" s="4"/>
+      <c r="K18" s="5"/>
+    </row>
+    <row r="19" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D19" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E19" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H18" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D19" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>49</v>
-      </c>
       <c r="F19" s="11" t="n">
-        <v>90</v>
+        <v>2.89</v>
       </c>
       <c r="G19" s="8" t="n">
         <f aca="false">D19*F19</f>
-        <v>90</v>
+        <v>11.56</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>17</v>
+      </c>
+      <c r="I19" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J19" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K19" s="5"/>
+    </row>
+    <row r="20" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="D20" s="9" t="n">
-        <v>2</v>
+        <v>66</v>
+      </c>
+      <c r="D20" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="F20" s="11" t="n">
-        <v>1.5</v>
+        <v>37</v>
+      </c>
+      <c r="F20" s="12" t="n">
+        <v>3</v>
       </c>
       <c r="G20" s="8" t="n">
         <f aca="false">D20*F20</f>
         <v>3</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>41</v>
+      </c>
+      <c r="I20" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J20" s="4"/>
+      <c r="K20" s="5"/>
+    </row>
+    <row r="21" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="D21" s="9" t="n">
-        <v>2</v>
+        <v>69</v>
+      </c>
+      <c r="D21" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="F21" s="11" t="n">
-        <v>2</v>
+        <v>70</v>
+      </c>
+      <c r="F21" s="12" t="n">
+        <v>90</v>
       </c>
       <c r="G21" s="8" t="n">
         <f aca="false">D21*F21</f>
-        <v>4</v>
+        <v>90</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>41</v>
+      </c>
+      <c r="I21" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="J21" s="4"/>
+      <c r="K21" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>54</v>
+        <v>73</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D22" s="9" t="n">
-        <v>1</v>
+        <v>74</v>
+      </c>
+      <c r="D22" s="10" t="n">
+        <v>2</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F22" s="11" t="n">
-        <v>10</v>
+        <v>16</v>
+      </c>
+      <c r="F22" s="12" t="n">
+        <v>1.5</v>
       </c>
       <c r="G22" s="8" t="n">
         <f aca="false">D22*F22</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>41</v>
+      </c>
+      <c r="I22" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="J22" s="4"/>
+      <c r="K22" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="D23" s="9" t="n">
-        <v>3</v>
+        <v>77</v>
+      </c>
+      <c r="D23" s="10" t="n">
+        <v>2</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F23" s="11" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="F23" s="12" t="n">
+        <v>2</v>
       </c>
       <c r="G23" s="8" t="n">
         <f aca="false">D23*F23</f>
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>41</v>
+      </c>
+      <c r="I23" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="J23" s="4"/>
+      <c r="K23" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="D24" s="9" t="n">
-        <v>2</v>
+        <v>79</v>
+      </c>
+      <c r="D24" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="F24" s="11" t="n">
-        <v>4</v>
+        <v>2.4</v>
       </c>
       <c r="G24" s="8" t="n">
         <f aca="false">D24*F24</f>
-        <v>8</v>
+        <v>2.4</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>17</v>
+      </c>
+      <c r="I24" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J24" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K24" s="5"/>
+    </row>
+    <row r="25" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>62</v>
+        <v>80</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="D25" s="9" t="n">
+        <v>81</v>
+      </c>
+      <c r="D25" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>20</v>
+        <v>2.5</v>
       </c>
       <c r="G25" s="8" t="n">
         <f aca="false">D25*F25</f>
-        <v>20</v>
+        <v>2.5</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>17</v>
+      </c>
+      <c r="I25" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="J25" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K25" s="5"/>
+    </row>
+    <row r="26" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D26" s="9" t="n">
+        <v>84</v>
+      </c>
+      <c r="D26" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="F26" s="11" t="n">
-        <v>30</v>
+        <v>85</v>
+      </c>
+      <c r="F26" s="12" t="n">
+        <v>10</v>
       </c>
       <c r="G26" s="8" t="n">
         <f aca="false">D26*F26</f>
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F28" s="12" t="s">
-        <v>67</v>
+        <v>41</v>
+      </c>
+      <c r="I26" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="J26" s="4"/>
+      <c r="K26" s="5"/>
+    </row>
+    <row r="27" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="D27" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F27" s="11" t="n">
+        <v>8.55</v>
+      </c>
+      <c r="G27" s="8" t="n">
+        <f aca="false">D27*F27</f>
+        <v>25.65</v>
+      </c>
+      <c r="H27" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I27" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J27" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K27" s="5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="D28" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F28" s="11" t="n">
+        <v>1.05</v>
       </c>
       <c r="G28" s="8" t="n">
-        <f aca="false">SUMIFS(G5:G26,H5:H26,"fornito da te")+SUMIFS(G5:G26,H5:H26,"OBI, verificato 18/10/2026")</f>
-        <v>259.99</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F29" s="12" t="s">
-        <v>68</v>
+        <f aca="false">D28*F28</f>
+        <v>1.05</v>
+      </c>
+      <c r="H28" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I28" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J28" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K28" s="5"/>
+    </row>
+    <row r="29" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="D29" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F29" s="12" t="n">
+        <v>20</v>
       </c>
       <c r="G29" s="8" t="n">
-        <f aca="false">SUMIFS(G5:G26,H5:H26,"stima – da verificare")</f>
-        <v>362.7</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F30" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="G30" s="14" t="n">
-        <f aca="false">SUM(G5:G26)</f>
-        <v>622.69</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F32" s="12" t="s">
-        <v>70</v>
+        <f aca="false">D29*F29</f>
+        <v>20</v>
+      </c>
+      <c r="H29" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="I29" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J29" s="4"/>
+      <c r="K29" s="5"/>
+    </row>
+    <row r="30" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="D30" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F30" s="11" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="G30" s="8" t="n">
+        <f aca="false">D30*F30</f>
+        <v>27.9</v>
+      </c>
+      <c r="H30" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I30" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J30" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K30" s="5"/>
+    </row>
+    <row r="31" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="D31" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F31" s="11" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="G31" s="8" t="n">
+        <f aca="false">D31*F31</f>
+        <v>6.7</v>
+      </c>
+      <c r="H31" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I31" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J31" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K31" s="5"/>
+    </row>
+    <row r="32" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="D32" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="F32" s="12" t="n">
+        <v>8</v>
       </c>
       <c r="G32" s="8" t="n">
-        <f aca="false">SUMIFS(G5:G26,A5:A26,"Legno")</f>
-        <v>269.99</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F33" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="G33" s="8" t="n">
-        <f aca="false">SUMIFS(G5:G26,A5:A26,"Ferramenta telaio")</f>
-        <v>142.7</v>
-      </c>
+        <f aca="false">D32*F32</f>
+        <v>8</v>
+      </c>
+      <c r="H32" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="I32" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J32" s="4"/>
+      <c r="K32" s="5"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F34" s="12" t="s">
-        <v>72</v>
+      <c r="F34" s="13" t="s">
+        <v>101</v>
       </c>
       <c r="G34" s="8" t="n">
-        <f aca="false">SUMIFS(G5:G26,A5:A26,"Zona ricarica")</f>
+        <f aca="false">SUMIFS(G5:G32,H5:H32,"verificato 18/10/2026")</f>
+        <v>429.88</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F35" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="G35" s="8" t="n">
+        <f aca="false">SUMIFS(G5:G32,H5:H32,"stima – da verificare")</f>
+        <v>183.4</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F36" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="G36" s="15" t="n">
+        <f aca="false">SUM(G5:G32)</f>
+        <v>613.28</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F38" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="G38" s="8" t="n">
+        <f aca="false">SUMIFS(G5:G32,A5:A32,"Legno")</f>
+        <v>262.2</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F39" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="G39" s="8" t="n">
+        <f aca="false">SUMIFS(G5:G32,A5:A32,"Ferramenta telaio")</f>
+        <v>149.88</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F40" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="G40" s="8" t="n">
+        <f aca="false">SUMIFS(G5:G32,A5:A32,"Zona ricarica")</f>
+        <v>111.9</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F41" s="13" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F35" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="G35" s="8" t="n">
-        <f aca="false">SUMIFS(G5:G26,A5:A26,"Elettrico")</f>
-        <v>73</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F36" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="G36" s="8" t="n">
-        <f aca="false">SUMIFS(G5:G26,A5:A26,"Finitura")</f>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="2" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="2" t="s">
-        <v>76</v>
+      <c r="G41" s="8" t="n">
+        <f aca="false">SUMIFS(G5:G32,A5:A32,"Elettrico")</f>
+        <v>46.7</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F42" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="G42" s="8" t="n">
+        <f aca="false">SUMIFS(G5:G32,A5:A32,"Finitura")</f>
+        <v>42.6</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F44" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="G44" s="8" t="n">
+        <f aca="false">SUMIFS(G5:G32,I5:I32,"Leroy Merlin")</f>
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F45" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="G45" s="8" t="n">
+        <f aca="false">SUMIFS(G5:G32,I5:I32,"OBI")</f>
+        <v>80.28</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F46" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="G46" s="8" t="n">
+        <f aca="false">SUMIFS(G5:G32,I5:I32,"Tecnomat")</f>
+        <v>393.1</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F47" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="G47" s="8" t="n">
+        <f aca="false">SUMIFS(G5:G32,I5:I32,"ferramenta/online")</f>
+        <v>47.4</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F48" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="G48" s="8" t="n">
+        <f aca="false">SUMIFS(G5:G32,I5:I32,"officina/carpenteria")</f>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="2" t="s">
+        <v>116</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="J5" r:id="rId1" display="apri"/>
+    <hyperlink ref="J6" r:id="rId2" display="apri"/>
+    <hyperlink ref="J7" r:id="rId3" display="apri"/>
+    <hyperlink ref="J8" r:id="rId4" display="apri"/>
+    <hyperlink ref="J9" r:id="rId5" display="apri"/>
+    <hyperlink ref="J10" r:id="rId6" display="apri"/>
+    <hyperlink ref="J12" r:id="rId7" display="apri"/>
+    <hyperlink ref="J13" r:id="rId8" display="apri"/>
+    <hyperlink ref="J14" r:id="rId9" display="apri"/>
+    <hyperlink ref="J15" r:id="rId10" display="apri"/>
+    <hyperlink ref="J16" r:id="rId11" display="apri"/>
+    <hyperlink ref="J17" r:id="rId12" display="apri"/>
+    <hyperlink ref="J19" r:id="rId13" display="apri"/>
+    <hyperlink ref="J24" r:id="rId14" display="apri"/>
+    <hyperlink ref="J25" r:id="rId15" display="apri"/>
+    <hyperlink ref="J27" r:id="rId16" display="apri"/>
+    <hyperlink ref="J28" r:id="rId17" display="apri"/>
+    <hyperlink ref="J30" r:id="rId18" display="apri"/>
+    <hyperlink ref="J31" r:id="rId19" display="apri"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1715,63 +2282,63 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>77</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>78</v>
+        <v>118</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>79</v>
+        <v>119</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>81</v>
+        <v>121</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>82</v>
+        <v>122</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>83</v>
+        <v>123</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>84</v>
+        <v>124</v>
       </c>
       <c r="H4" s="3"/>
       <c r="I4" s="3" t="s">
-        <v>85</v>
+        <v>125</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>86</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>87</v>
+        <v>127</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="C5" s="15" t="n">
+        <v>128</v>
+      </c>
+      <c r="C5" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="D5" s="10" t="n">
+      <c r="D5" s="11" t="n">
         <v>83.5</v>
       </c>
-      <c r="E5" s="16" t="n">
+      <c r="E5" s="17" t="n">
         <f aca="false">D5/C5</f>
         <v>13.9166666666667</v>
       </c>
-      <c r="F5" s="17" t="n">
+      <c r="F5" s="18" t="n">
         <v>15.26</v>
       </c>
-      <c r="G5" s="15" t="n">
+      <c r="G5" s="16" t="n">
         <v>5.1</v>
       </c>
-      <c r="I5" s="9" t="n">
+      <c r="I5" s="10" t="n">
         <v>3</v>
       </c>
       <c r="J5" s="8" t="n">
@@ -1781,28 +2348,28 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>89</v>
+        <v>129</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="C6" s="15" t="n">
+        <v>128</v>
+      </c>
+      <c r="C6" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="D6" s="10" t="n">
+      <c r="D6" s="11" t="n">
         <v>55.9</v>
       </c>
-      <c r="E6" s="16" t="n">
+      <c r="E6" s="17" t="n">
         <f aca="false">D6/C6</f>
         <v>13.975</v>
       </c>
-      <c r="F6" s="17" t="n">
+      <c r="F6" s="18" t="n">
         <v>15.26</v>
       </c>
-      <c r="G6" s="15" t="n">
+      <c r="G6" s="16" t="n">
         <v>5.1</v>
       </c>
-      <c r="I6" s="9" t="n">
+      <c r="I6" s="10" t="n">
         <v>4</v>
       </c>
       <c r="J6" s="8" t="n">
@@ -1812,28 +2379,28 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>90</v>
+        <v>130</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="C7" s="15" t="n">
+        <v>131</v>
+      </c>
+      <c r="C7" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="D7" s="10" t="n">
+      <c r="D7" s="11" t="n">
         <v>31.9</v>
       </c>
-      <c r="E7" s="16" t="n">
+      <c r="E7" s="17" t="n">
         <f aca="false">D7/C7</f>
         <v>7.975</v>
       </c>
-      <c r="F7" s="17" t="n">
+      <c r="F7" s="18" t="n">
         <v>16.22</v>
       </c>
-      <c r="G7" s="15" t="n">
+      <c r="G7" s="16" t="n">
         <v>1.6</v>
       </c>
-      <c r="I7" s="9" t="n">
+      <c r="I7" s="10" t="n">
         <v>5</v>
       </c>
       <c r="J7" s="8" t="n">
@@ -1842,61 +2409,61 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="s">
-        <v>92</v>
-      </c>
-      <c r="B8" s="19" t="s">
-        <v>93</v>
-      </c>
-      <c r="C8" s="20" t="n">
+      <c r="A8" s="19" t="s">
+        <v>132</v>
+      </c>
+      <c r="B8" s="20" t="s">
+        <v>133</v>
+      </c>
+      <c r="C8" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="D8" s="21" t="n">
+      <c r="D8" s="22" t="n">
         <v>29.9</v>
       </c>
-      <c r="E8" s="22" t="n">
+      <c r="E8" s="23" t="n">
         <f aca="false">D8/C8</f>
         <v>7.475</v>
       </c>
-      <c r="F8" s="23" t="n">
+      <c r="F8" s="24" t="n">
         <v>15.9</v>
       </c>
-      <c r="G8" s="20" t="n">
+      <c r="G8" s="21" t="n">
         <v>3.4</v>
       </c>
-      <c r="H8" s="24"/>
-      <c r="I8" s="25" t="n">
+      <c r="H8" s="25"/>
+      <c r="I8" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="J8" s="26" t="n">
+      <c r="J8" s="27" t="n">
         <f aca="false">I8*D8</f>
         <v>149.5</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>94</v>
+        <v>134</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="C9" s="15" t="n">
+        <v>135</v>
+      </c>
+      <c r="C9" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="D9" s="10" t="n">
+      <c r="D9" s="11" t="n">
         <v>39.9</v>
       </c>
-      <c r="E9" s="16" t="n">
+      <c r="E9" s="17" t="n">
         <f aca="false">D9/C9</f>
         <v>9.975</v>
       </c>
-      <c r="F9" s="17" t="n">
+      <c r="F9" s="18" t="n">
         <v>15.58</v>
       </c>
-      <c r="G9" s="15" t="n">
+      <c r="G9" s="16" t="n">
         <v>4.2</v>
       </c>
-      <c r="I9" s="9" t="n">
+      <c r="I9" s="10" t="n">
         <v>4</v>
       </c>
       <c r="J9" s="8" t="n">
@@ -1906,7 +2473,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>96</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -1925,138 +2492,159 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="70"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>99</v>
+        <v>138</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>101</v>
+        <v>139</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>102</v>
+        <v>140</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>7</v>
+        <v>141</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>103</v>
+        <v>142</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="18" t="s">
-        <v>106</v>
-      </c>
-      <c r="B5" s="19" t="s">
-        <v>107</v>
-      </c>
-      <c r="C5" s="19" t="s">
-        <v>108</v>
-      </c>
-      <c r="D5" s="25" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="B5" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="20" t="s">
+        <v>144</v>
+      </c>
+      <c r="D5" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="21" t="n">
-        <v>31.49</v>
-      </c>
-      <c r="F5" s="26" t="n">
+      <c r="E5" s="22" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="F5" s="27" t="n">
         <f aca="false">D5*E5</f>
-        <v>31.49</v>
-      </c>
-      <c r="G5" s="27" t="s">
-        <v>19</v>
-      </c>
-      <c r="H5" s="27" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>27.5</v>
+      </c>
+      <c r="G5" s="28" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>110</v>
+        <v>146</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>111</v>
+        <v>82</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="D6" s="9" t="n">
+        <v>144</v>
+      </c>
+      <c r="D6" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="10" t="n">
-        <v>79</v>
+      <c r="E6" s="11" t="n">
+        <v>30.5</v>
       </c>
       <c r="F6" s="8" t="n">
         <f aca="false">D6*E6</f>
-        <v>79</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>30.5</v>
+      </c>
+      <c r="G6" s="5"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>114</v>
+        <v>146</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>115</v>
+        <v>33</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="D7" s="9" t="n">
-        <v>14</v>
-      </c>
-      <c r="E7" s="10" t="n">
-        <v>8.19</v>
+        <v>144</v>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>31.49</v>
       </c>
       <c r="F7" s="8" t="n">
         <f aca="false">D7*E7</f>
+        <v>31.49</v>
+      </c>
+      <c r="G7" s="5"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>79</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <f aca="false">D8*E8</f>
+        <v>79</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="D9" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>8.19</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <f aca="false">D9*E9</f>
         <v>114.66</v>
       </c>
-      <c r="G7" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
-        <v>118</v>
+      <c r="G9" s="5" t="s">
+        <v>152</v>
       </c>
     </row>
   </sheetData>
@@ -2075,7 +2663,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -2085,101 +2673,101 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>119</v>
+        <v>153</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>120</v>
+        <v>154</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>121</v>
+        <v>155</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>122</v>
+        <v>156</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>123</v>
+        <v>157</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>124</v>
+        <v>158</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="C4" s="28" t="n">
+        <v>159</v>
+      </c>
+      <c r="C4" s="29" t="n">
         <v>3694</v>
       </c>
-      <c r="D4" s="29" t="n">
+      <c r="D4" s="30" t="n">
         <f aca="false">4000-C4</f>
         <v>306</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>126</v>
+        <v>160</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="C5" s="28" t="n">
+        <v>161</v>
+      </c>
+      <c r="C5" s="29" t="n">
         <v>3614</v>
       </c>
-      <c r="D5" s="29" t="n">
+      <c r="D5" s="30" t="n">
         <f aca="false">4000-C5</f>
         <v>386</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>128</v>
+        <v>162</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="C6" s="28" t="n">
+        <v>163</v>
+      </c>
+      <c r="C6" s="29" t="n">
         <v>3654</v>
       </c>
-      <c r="D6" s="29" t="n">
+      <c r="D6" s="30" t="n">
         <f aca="false">4000-C6</f>
         <v>346</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>130</v>
+        <v>164</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="C7" s="28" t="n">
+        <v>165</v>
+      </c>
+      <c r="C7" s="29" t="n">
         <v>1418</v>
       </c>
-      <c r="D7" s="29" t="n">
+      <c r="D7" s="30" t="n">
         <f aca="false">4000-C7</f>
         <v>2582</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>132</v>
+        <v>166</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="C8" s="28" t="n">
+        <v>167</v>
+      </c>
+      <c r="C8" s="29" t="n">
         <v>3686</v>
       </c>
-      <c r="D8" s="29" t="n">
+      <c r="D8" s="30" t="n">
         <f aca="false">4000-C8</f>
         <v>314</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
-        <v>134</v>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>168</v>
       </c>
     </row>
   </sheetData>

</xml_diff>